<commit_message>
Implemente el uso de OR-Tools en el scheduler.py con lo que se logra hacer un scheduler inicial
</commit_message>
<xml_diff>
--- a/data/sample_courses.xlsx
+++ b/data/sample_courses.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matit\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matit\Desktop\IAA Proyect\scheduler-mvp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F5488F4-8FFE-4933-9287-A378ABF8EEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEC6BDD-30E1-4DA8-9B13-76DDAAEE1BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="297">
   <si>
     <t>LLAVE Código- sec</t>
   </si>
@@ -1275,6 +1275,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="119.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="116.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="156" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="43.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="117.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="114.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="18" width="115" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1436,6 +1452,21 @@
       <c r="J4" t="s">
         <v>61</v>
       </c>
+      <c r="N4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P4" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1652,6 +1683,21 @@
       <c r="J10" t="s">
         <v>261</v>
       </c>
+      <c r="N10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O10" t="s">
+        <v>24</v>
+      </c>
+      <c r="P10" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>24</v>
+      </c>
+      <c r="R10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -2247,6 +2293,21 @@
       <c r="L24" t="s">
         <v>214</v>
       </c>
+      <c r="N24" t="s">
+        <v>24</v>
+      </c>
+      <c r="O24" t="s">
+        <v>24</v>
+      </c>
+      <c r="P24" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>24</v>
+      </c>
+      <c r="R24" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -2270,6 +2331,21 @@
       <c r="J25" t="s">
         <v>265</v>
       </c>
+      <c r="N25" t="s">
+        <v>24</v>
+      </c>
+      <c r="O25" t="s">
+        <v>24</v>
+      </c>
+      <c r="P25" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>24</v>
+      </c>
+      <c r="R25" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -2331,6 +2407,21 @@
       <c r="J27" t="s">
         <v>273</v>
       </c>
+      <c r="N27" t="s">
+        <v>24</v>
+      </c>
+      <c r="O27" t="s">
+        <v>24</v>
+      </c>
+      <c r="P27" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>24</v>
+      </c>
+      <c r="R27" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -2354,6 +2445,21 @@
       <c r="J28" t="s">
         <v>277</v>
       </c>
+      <c r="N28" t="s">
+        <v>24</v>
+      </c>
+      <c r="O28" t="s">
+        <v>24</v>
+      </c>
+      <c r="P28" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>24</v>
+      </c>
+      <c r="R28" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -2377,6 +2483,21 @@
       <c r="J29" t="s">
         <v>281</v>
       </c>
+      <c r="N29" t="s">
+        <v>24</v>
+      </c>
+      <c r="O29" t="s">
+        <v>24</v>
+      </c>
+      <c r="P29" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>24</v>
+      </c>
+      <c r="R29" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -3126,6 +3247,21 @@
       <c r="J48" t="s">
         <v>143</v>
       </c>
+      <c r="N48" t="s">
+        <v>24</v>
+      </c>
+      <c r="O48" t="s">
+        <v>24</v>
+      </c>
+      <c r="P48" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>24</v>
+      </c>
+      <c r="R48" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -3149,6 +3285,21 @@
       <c r="J49" t="s">
         <v>147</v>
       </c>
+      <c r="N49" t="s">
+        <v>24</v>
+      </c>
+      <c r="O49" t="s">
+        <v>24</v>
+      </c>
+      <c r="P49" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>24</v>
+      </c>
+      <c r="R49" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -3172,6 +3323,21 @@
       <c r="J50" t="s">
         <v>151</v>
       </c>
+      <c r="N50" t="s">
+        <v>24</v>
+      </c>
+      <c r="O50" t="s">
+        <v>24</v>
+      </c>
+      <c r="P50" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>24</v>
+      </c>
+      <c r="R50" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
@@ -3194,6 +3360,21 @@
       </c>
       <c r="J51" t="s">
         <v>155</v>
+      </c>
+      <c r="N51" t="s">
+        <v>24</v>
+      </c>
+      <c r="O51" t="s">
+        <v>24</v>
+      </c>
+      <c r="P51" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>24</v>
+      </c>
+      <c r="R51" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.25">

</xml_diff>